<commit_message>
Preserve BAS account metadata in XLSX conversion
</commit_message>
<xml_diff>
--- a/src/main/resources/account/default/BAS-2026---Aktiebolag.xlsx
+++ b/src/main/resources/account/default/BAS-2026---Aktiebolag.xlsx
@@ -427,6 +427,9 @@
           <t>BAS 2026 - Aktiebolag</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +442,9 @@
           <t>EUBAS97</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +457,9 @@
           <t>2026</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -461,6 +470,9 @@
       <c r="B4" t="n">
         <v>6</v>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2776,7 +2788,11 @@
           <t>Pågående arbeten, nedlagda kostnader</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D140" t="inlineStr">
         <is>
           <t>7245</t>
@@ -6406,7 +6422,11 @@
           <t>Kortfristiga lån från kreditinstitut</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr"/>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D362" t="inlineStr">
         <is>
           <t>7361</t>
@@ -6423,7 +6443,11 @@
           <t>Byggnadskreditiv, kortfristig del</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr"/>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D363" t="inlineStr">
         <is>
           <t>7361</t>
@@ -6491,7 +6515,11 @@
           <t>Ej inlösta presentkort</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr"/>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
       <c r="D367" t="inlineStr">
         <is>
           <t>7362</t>
@@ -6542,7 +6570,11 @@
           <t>Pågående arbeten, fakturering</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr"/>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
       <c r="D370" t="inlineStr">
         <is>
           <t>7363</t>
@@ -7031,7 +7063,11 @@
           <t>Utgående moms, 25 %</t>
         </is>
       </c>
-      <c r="C399" t="inlineStr"/>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D399" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7048,7 +7084,11 @@
           <t>Utgående moms på försäljning inom Sverige, 25 %</t>
         </is>
       </c>
-      <c r="C400" t="inlineStr"/>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D400" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7065,7 +7105,11 @@
           <t>Utgående moms på egna uttag, 25 %</t>
         </is>
       </c>
-      <c r="C401" t="inlineStr"/>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D401" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7082,7 +7126,11 @@
           <t>Utgående moms för uthyrning, 25 %</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr"/>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D402" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7099,7 +7147,11 @@
           <t>Utgående moms omvänd betalskyldighet, 25 %</t>
         </is>
       </c>
-      <c r="C403" t="inlineStr"/>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>U1MI</t>
+        </is>
+      </c>
       <c r="D403" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7116,7 +7168,11 @@
           <t>Utgående moms import av varor, 25 %</t>
         </is>
       </c>
-      <c r="C404" t="inlineStr"/>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>U1MI</t>
+        </is>
+      </c>
       <c r="D404" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7150,7 +7206,11 @@
           <t>Vilande utgående moms, 25 %</t>
         </is>
       </c>
-      <c r="C406" t="inlineStr"/>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
       <c r="D406" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7184,7 +7244,11 @@
           <t>Utgående moms på försäljning inom Sverige, 12 %</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr"/>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
       <c r="D408" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7201,7 +7265,11 @@
           <t>Utgående moms på egna uttag, 12 %</t>
         </is>
       </c>
-      <c r="C409" t="inlineStr"/>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
       <c r="D409" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7235,7 +7303,11 @@
           <t>Utgående moms omvänd betalningsskyldighet 12 %</t>
         </is>
       </c>
-      <c r="C411" t="inlineStr"/>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>U2MI</t>
+        </is>
+      </c>
       <c r="D411" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7252,7 +7324,11 @@
           <t>Utgående moms import av varor, 12 %</t>
         </is>
       </c>
-      <c r="C412" t="inlineStr"/>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>U2MI</t>
+        </is>
+      </c>
       <c r="D412" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7286,7 +7362,11 @@
           <t>Vilande utgående moms, 12 %</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr"/>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
       <c r="D414" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7320,7 +7400,11 @@
           <t>Utgående moms på försäljning inom Sverige, 6 %</t>
         </is>
       </c>
-      <c r="C416" t="inlineStr"/>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
       <c r="D416" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7337,7 +7421,11 @@
           <t>Utgående moms på egna uttag, 6 %</t>
         </is>
       </c>
-      <c r="C417" t="inlineStr"/>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
       <c r="D417" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7371,7 +7459,11 @@
           <t>Utgående moms omvänd betalningsskyldighet, 6 %</t>
         </is>
       </c>
-      <c r="C419" t="inlineStr"/>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>U3MI</t>
+        </is>
+      </c>
       <c r="D419" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7388,7 +7480,11 @@
           <t>Utgående moms import av varor, 6 %</t>
         </is>
       </c>
-      <c r="C420" t="inlineStr"/>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>U3MI</t>
+        </is>
+      </c>
       <c r="D420" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7422,7 +7518,11 @@
           <t>Vilande utgående moms, 6 %</t>
         </is>
       </c>
-      <c r="C422" t="inlineStr"/>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>U3</t>
+        </is>
+      </c>
       <c r="D422" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7439,7 +7539,11 @@
           <t>Ingående moms</t>
         </is>
       </c>
-      <c r="C423" t="inlineStr"/>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D423" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7456,7 +7560,11 @@
           <t>Debiterad ingående moms</t>
         </is>
       </c>
-      <c r="C424" t="inlineStr"/>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D424" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7473,7 +7581,11 @@
           <t>Debiterad ingående moms i anslutning till frivillig betalningsskyldighet</t>
         </is>
       </c>
-      <c r="C425" t="inlineStr"/>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D425" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7490,7 +7602,11 @@
           <t>Beräknad ingående moms på förvärv från utlandet</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr"/>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D426" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7507,7 +7623,11 @@
           <t>Ingående moms på uthyrning</t>
         </is>
       </c>
-      <c r="C427" t="inlineStr"/>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D427" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7541,7 +7661,11 @@
           <t>Vilande ingående moms</t>
         </is>
       </c>
-      <c r="C429" t="inlineStr"/>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D429" t="inlineStr">
         <is>
           <t>7369</t>
@@ -7558,7 +7682,11 @@
           <t>Ingående moms, blandad verksamhet</t>
         </is>
       </c>
-      <c r="C430" t="inlineStr"/>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="D430" t="inlineStr">
         <is>
           <t>7369</t>
@@ -9246,7 +9374,11 @@
           <t>Fakturerade kostnader (gruppkonto)</t>
         </is>
       </c>
-      <c r="C530" t="inlineStr"/>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D530" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9263,7 +9395,11 @@
           <t>Fakturerat emballage</t>
         </is>
       </c>
-      <c r="C531" t="inlineStr"/>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D531" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9314,7 +9450,11 @@
           <t>Fakturerade frakter</t>
         </is>
       </c>
-      <c r="C534" t="inlineStr"/>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D534" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9348,7 +9488,11 @@
           <t>Fakturerade frakter, export</t>
         </is>
       </c>
-      <c r="C536" t="inlineStr"/>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>VTEU</t>
+        </is>
+      </c>
       <c r="D536" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9365,7 +9509,11 @@
           <t>Fakturerade tull- och  speditionskostnader m.m.</t>
         </is>
       </c>
-      <c r="C537" t="inlineStr"/>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="D537" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9382,7 +9530,11 @@
           <t>Faktureringsavgifter</t>
         </is>
       </c>
-      <c r="C538" t="inlineStr"/>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D538" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9399,7 +9551,11 @@
           <t>Faktureringsavgifter, EU-land</t>
         </is>
       </c>
-      <c r="C539" t="inlineStr"/>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="D539" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9416,7 +9572,11 @@
           <t>Faktureringsavgifter, export</t>
         </is>
       </c>
-      <c r="C540" t="inlineStr"/>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>VTEU</t>
+        </is>
+      </c>
       <c r="D540" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9433,7 +9593,11 @@
           <t>Fakturerade resekostnader</t>
         </is>
       </c>
-      <c r="C541" t="inlineStr"/>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D541" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9450,7 +9614,11 @@
           <t>Fakturerade kostnader till  koncernföretag</t>
         </is>
       </c>
-      <c r="C542" t="inlineStr"/>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D542" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9518,7 +9686,11 @@
           <t>Fakturerade kostnader till  intresseföretag, gemensamt styrda företag och övriga företag som det finns ett ägarintresse i</t>
         </is>
       </c>
-      <c r="C546" t="inlineStr"/>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D546" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9535,7 +9707,11 @@
           <t>Övriga fakturerade kostnader</t>
         </is>
       </c>
-      <c r="C547" t="inlineStr"/>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D547" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9552,7 +9728,11 @@
           <t>Rörelsens sidointäkter (gruppkonto)</t>
         </is>
       </c>
-      <c r="C548" t="inlineStr"/>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D548" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9569,7 +9749,11 @@
           <t>Försäljning av material</t>
         </is>
       </c>
-      <c r="C549" t="inlineStr"/>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D549" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9654,7 +9838,11 @@
           <t>Tillfällig uthyrning av personal</t>
         </is>
       </c>
-      <c r="C554" t="inlineStr"/>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D554" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9773,7 +9961,11 @@
           <t>Övriga sidointäkter</t>
         </is>
       </c>
-      <c r="C561" t="inlineStr"/>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D561" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9790,7 +9982,11 @@
           <t>Intäktskorrigeringar (gruppkonto)</t>
         </is>
       </c>
-      <c r="C562" t="inlineStr"/>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D562" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9807,7 +10003,11 @@
           <t>Ofördelade intäktsreduktioner</t>
         </is>
       </c>
-      <c r="C563" t="inlineStr"/>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D563" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9824,7 +10024,11 @@
           <t>Lämnade rabatter</t>
         </is>
       </c>
-      <c r="C564" t="inlineStr"/>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D564" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9896,7 +10100,11 @@
           <t>Punktskatter</t>
         </is>
       </c>
-      <c r="C568" t="inlineStr"/>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D568" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9947,7 +10155,11 @@
           <t>Övriga intäktskorrigeringar</t>
         </is>
       </c>
-      <c r="C571" t="inlineStr"/>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D571" t="inlineStr">
         <is>
           <t>7410</t>
@@ -9998,7 +10210,11 @@
           <t>Aktiverat arbete (omkostnader)</t>
         </is>
       </c>
-      <c r="C574" t="inlineStr"/>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
       <c r="D574" t="inlineStr">
         <is>
           <t>7412</t>
@@ -10032,7 +10248,11 @@
           <t>Övriga rörelseintäkter (gruppkonto)</t>
         </is>
       </c>
-      <c r="C576" t="inlineStr"/>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>MP1</t>
+        </is>
+      </c>
       <c r="D576" t="inlineStr">
         <is>
           <t>7413</t>
@@ -10219,7 +10439,11 @@
           <t>Återvunna, tidigare avskrivna  kundfordringar</t>
         </is>
       </c>
-      <c r="C587" t="inlineStr"/>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
       <c r="D587" t="inlineStr">
         <is>
           <t>7413</t>
@@ -10321,7 +10545,11 @@
           <t>Erhållna offentliga bidrag</t>
         </is>
       </c>
-      <c r="C593" t="inlineStr"/>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
       <c r="D593" t="inlineStr">
         <is>
           <t>7413</t>
@@ -10423,7 +10651,11 @@
           <t>Övriga ersättningar, bidrag och  intäkter</t>
         </is>
       </c>
-      <c r="C599" t="inlineStr"/>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
       <c r="D599" t="inlineStr">
         <is>
           <t>7413</t>

</xml_diff>